<commit_message>
LeetCode Problem No 1 - Two Sum
</commit_message>
<xml_diff>
--- a/leetcode_tracker.xlsx
+++ b/leetcode_tracker.xlsx
@@ -1,18 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\Desktop\DSA\LeetCode\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783123DB-A73C-487E-AD05-C067ADC738C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Log" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Log" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -23,102 +37,98 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
-    <t xml:space="preserve">Date Solved</t>
+    <t>Date Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">Problem #</t>
+    <t>Problem #</t>
   </si>
   <si>
-    <t xml:space="preserve">Problem Name</t>
+    <t>Problem Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Difficulty</t>
+    <t>Difficulty</t>
   </si>
   <si>
-    <t xml:space="preserve">Topic/Tags</t>
+    <t>Topic/Tags</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
+    <t>Status</t>
   </si>
   <si>
-    <t xml:space="preserve">Language</t>
+    <t>Language</t>
   </si>
   <si>
-    <t xml:space="preserve">Time Taken (min)</t>
+    <t>Time Taken (min)</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempts</t>
+    <t>Attempts</t>
   </si>
   <si>
-    <t xml:space="preserve">Solution Link</t>
+    <t>Solution Link</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes</t>
+    <t>Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-30</t>
+    <t>2026-07-30</t>
   </si>
   <si>
-    <t xml:space="preserve">1</t>
+    <t>1</t>
   </si>
   <si>
-    <t xml:space="preserve">Two Sum</t>
+    <t>Two Sum</t>
   </si>
   <si>
-    <t xml:space="preserve">Easy</t>
+    <t>Easy</t>
   </si>
   <si>
-    <t xml:space="preserve">Array, Hash Map</t>
+    <t>Array, Hash Map</t>
   </si>
   <si>
-    <t xml:space="preserve">Solved</t>
+    <t>Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">Python</t>
+    <t>Python</t>
   </si>
   <si>
-    <t xml:space="preserve">https://github.com/yourname/leetcode/1-two-sum</t>
+    <t>https://github.com/yourname/leetcode/1-two-sum</t>
   </si>
   <si>
-    <t xml:space="preserve">Used a hash map for O(n); revisit for O(1) space follow-up</t>
+    <t>Used a hash map for O(n); revisit for O(1) space follow-up</t>
   </si>
   <si>
-    <t xml:space="preserve">LeetCode Progress Summary</t>
+    <t>LeetCode Progress Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Problems Logged</t>
+    <t>Total Problems Logged</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempted (not yet solved)</t>
+    <t>Attempted (not yet solved)</t>
   </si>
   <si>
-    <t xml:space="preserve">To Revisit</t>
+    <t>To Revisit</t>
   </si>
   <si>
-    <t xml:space="preserve">Bookmarked</t>
+    <t>Bookmarked</t>
   </si>
   <si>
-    <t xml:space="preserve">Easy Solved</t>
+    <t>Easy Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">Medium Solved</t>
+    <t>Medium Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">Hard Solved</t>
+    <t>Hard Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">Avg Time per Solve (min)</t>
+    <t>Avg Time per Solve (min)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-  </numFmts>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,55 +137,35 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF808080"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="14"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -193,14 +183,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFB7B7B7"/>
       </left>
@@ -216,69 +206,30 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -337,47 +288,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF305496"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -385,12 +352,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -419,7 +386,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -440,7 +407,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -491,7 +458,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -509,104 +476,103 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K200"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="30"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="11" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:11" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="6">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="6">
         <v>1</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -619,7 +585,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -632,7 +598,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -645,7 +611,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -658,7 +624,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -671,7 +637,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -684,7 +650,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -697,7 +663,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -710,7 +676,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -723,7 +689,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -736,7 +702,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -749,7 +715,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -762,7 +728,7 @@
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -775,7 +741,7 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -788,7 +754,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -801,7 +767,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -814,7 +780,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -827,7 +793,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -840,7 +806,7 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -853,7 +819,7 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -866,7 +832,7 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -879,7 +845,7 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -892,7 +858,7 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -905,7 +871,7 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -918,7 +884,7 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -931,7 +897,7 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -944,7 +910,7 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -957,7 +923,7 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -970,7 +936,7 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -983,7 +949,7 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -996,7 +962,7 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1009,7 +975,7 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1022,7 +988,7 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1035,7 +1001,7 @@
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1048,7 +1014,7 @@
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1061,7 +1027,7 @@
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1074,7 +1040,7 @@
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1087,7 +1053,7 @@
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1100,7 +1066,7 @@
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1113,7 +1079,7 @@
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1126,7 +1092,7 @@
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1139,7 +1105,7 @@
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1152,7 +1118,7 @@
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1165,7 +1131,7 @@
       <c r="J45" s="3"/>
       <c r="K45" s="3"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1178,7 +1144,7 @@
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1191,7 +1157,7 @@
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1204,7 +1170,7 @@
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1217,7 +1183,7 @@
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1230,7 +1196,7 @@
       <c r="J50" s="3"/>
       <c r="K50" s="3"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1243,7 +1209,7 @@
       <c r="J51" s="3"/>
       <c r="K51" s="3"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1256,7 +1222,7 @@
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1269,7 +1235,7 @@
       <c r="J53" s="3"/>
       <c r="K53" s="3"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1282,7 +1248,7 @@
       <c r="J54" s="3"/>
       <c r="K54" s="3"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1295,7 +1261,7 @@
       <c r="J55" s="3"/>
       <c r="K55" s="3"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1308,7 +1274,7 @@
       <c r="J56" s="3"/>
       <c r="K56" s="3"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1321,7 +1287,7 @@
       <c r="J57" s="3"/>
       <c r="K57" s="3"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1334,7 +1300,7 @@
       <c r="J58" s="3"/>
       <c r="K58" s="3"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1347,7 +1313,7 @@
       <c r="J59" s="3"/>
       <c r="K59" s="3"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1360,7 +1326,7 @@
       <c r="J60" s="3"/>
       <c r="K60" s="3"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1373,7 +1339,7 @@
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -1386,7 +1352,7 @@
       <c r="J62" s="3"/>
       <c r="K62" s="3"/>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1399,7 +1365,7 @@
       <c r="J63" s="3"/>
       <c r="K63" s="3"/>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -1412,7 +1378,7 @@
       <c r="J64" s="3"/>
       <c r="K64" s="3"/>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1425,7 +1391,7 @@
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -1438,7 +1404,7 @@
       <c r="J66" s="3"/>
       <c r="K66" s="3"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1451,7 +1417,7 @@
       <c r="J67" s="3"/>
       <c r="K67" s="3"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -1464,7 +1430,7 @@
       <c r="J68" s="3"/>
       <c r="K68" s="3"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1477,7 +1443,7 @@
       <c r="J69" s="3"/>
       <c r="K69" s="3"/>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -1490,7 +1456,7 @@
       <c r="J70" s="3"/>
       <c r="K70" s="3"/>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1503,7 +1469,7 @@
       <c r="J71" s="3"/>
       <c r="K71" s="3"/>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -1516,7 +1482,7 @@
       <c r="J72" s="3"/>
       <c r="K72" s="3"/>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -1529,7 +1495,7 @@
       <c r="J73" s="3"/>
       <c r="K73" s="3"/>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -1542,7 +1508,7 @@
       <c r="J74" s="3"/>
       <c r="K74" s="3"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -1555,7 +1521,7 @@
       <c r="J75" s="3"/>
       <c r="K75" s="3"/>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -1568,7 +1534,7 @@
       <c r="J76" s="3"/>
       <c r="K76" s="3"/>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -1581,7 +1547,7 @@
       <c r="J77" s="3"/>
       <c r="K77" s="3"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -1594,7 +1560,7 @@
       <c r="J78" s="3"/>
       <c r="K78" s="3"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -1607,7 +1573,7 @@
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -1620,7 +1586,7 @@
       <c r="J80" s="3"/>
       <c r="K80" s="3"/>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -1633,7 +1599,7 @@
       <c r="J81" s="3"/>
       <c r="K81" s="3"/>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -1646,7 +1612,7 @@
       <c r="J82" s="3"/>
       <c r="K82" s="3"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -1659,7 +1625,7 @@
       <c r="J83" s="3"/>
       <c r="K83" s="3"/>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -1672,7 +1638,7 @@
       <c r="J84" s="3"/>
       <c r="K84" s="3"/>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -1685,7 +1651,7 @@
       <c r="J85" s="3"/>
       <c r="K85" s="3"/>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -1698,7 +1664,7 @@
       <c r="J86" s="3"/>
       <c r="K86" s="3"/>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -1711,7 +1677,7 @@
       <c r="J87" s="3"/>
       <c r="K87" s="3"/>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -1724,7 +1690,7 @@
       <c r="J88" s="3"/>
       <c r="K88" s="3"/>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -1737,7 +1703,7 @@
       <c r="J89" s="3"/>
       <c r="K89" s="3"/>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -1750,7 +1716,7 @@
       <c r="J90" s="3"/>
       <c r="K90" s="3"/>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -1763,7 +1729,7 @@
       <c r="J91" s="3"/>
       <c r="K91" s="3"/>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -1776,7 +1742,7 @@
       <c r="J92" s="3"/>
       <c r="K92" s="3"/>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -1789,7 +1755,7 @@
       <c r="J93" s="3"/>
       <c r="K93" s="3"/>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -1802,7 +1768,7 @@
       <c r="J94" s="3"/>
       <c r="K94" s="3"/>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -1815,7 +1781,7 @@
       <c r="J95" s="3"/>
       <c r="K95" s="3"/>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -1828,7 +1794,7 @@
       <c r="J96" s="3"/>
       <c r="K96" s="3"/>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -1841,7 +1807,7 @@
       <c r="J97" s="3"/>
       <c r="K97" s="3"/>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -1854,7 +1820,7 @@
       <c r="J98" s="3"/>
       <c r="K98" s="3"/>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -1867,7 +1833,7 @@
       <c r="J99" s="3"/>
       <c r="K99" s="3"/>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -1880,7 +1846,7 @@
       <c r="J100" s="3"/>
       <c r="K100" s="3"/>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -1893,7 +1859,7 @@
       <c r="J101" s="3"/>
       <c r="K101" s="3"/>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -1906,7 +1872,7 @@
       <c r="J102" s="3"/>
       <c r="K102" s="3"/>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -1919,7 +1885,7 @@
       <c r="J103" s="3"/>
       <c r="K103" s="3"/>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -1932,7 +1898,7 @@
       <c r="J104" s="3"/>
       <c r="K104" s="3"/>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -1945,7 +1911,7 @@
       <c r="J105" s="3"/>
       <c r="K105" s="3"/>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -1958,7 +1924,7 @@
       <c r="J106" s="3"/>
       <c r="K106" s="3"/>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -1971,7 +1937,7 @@
       <c r="J107" s="3"/>
       <c r="K107" s="3"/>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -1984,7 +1950,7 @@
       <c r="J108" s="3"/>
       <c r="K108" s="3"/>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -1997,7 +1963,7 @@
       <c r="J109" s="3"/>
       <c r="K109" s="3"/>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -2010,7 +1976,7 @@
       <c r="J110" s="3"/>
       <c r="K110" s="3"/>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -2023,7 +1989,7 @@
       <c r="J111" s="3"/>
       <c r="K111" s="3"/>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -2036,7 +2002,7 @@
       <c r="J112" s="3"/>
       <c r="K112" s="3"/>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -2049,7 +2015,7 @@
       <c r="J113" s="3"/>
       <c r="K113" s="3"/>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -2062,7 +2028,7 @@
       <c r="J114" s="3"/>
       <c r="K114" s="3"/>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -2075,7 +2041,7 @@
       <c r="J115" s="3"/>
       <c r="K115" s="3"/>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -2088,7 +2054,7 @@
       <c r="J116" s="3"/>
       <c r="K116" s="3"/>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -2101,7 +2067,7 @@
       <c r="J117" s="3"/>
       <c r="K117" s="3"/>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -2114,7 +2080,7 @@
       <c r="J118" s="3"/>
       <c r="K118" s="3"/>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -2127,7 +2093,7 @@
       <c r="J119" s="3"/>
       <c r="K119" s="3"/>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -2140,7 +2106,7 @@
       <c r="J120" s="3"/>
       <c r="K120" s="3"/>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -2153,7 +2119,7 @@
       <c r="J121" s="3"/>
       <c r="K121" s="3"/>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -2166,7 +2132,7 @@
       <c r="J122" s="3"/>
       <c r="K122" s="3"/>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -2179,7 +2145,7 @@
       <c r="J123" s="3"/>
       <c r="K123" s="3"/>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -2192,7 +2158,7 @@
       <c r="J124" s="3"/>
       <c r="K124" s="3"/>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -2205,7 +2171,7 @@
       <c r="J125" s="3"/>
       <c r="K125" s="3"/>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -2218,7 +2184,7 @@
       <c r="J126" s="3"/>
       <c r="K126" s="3"/>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -2231,7 +2197,7 @@
       <c r="J127" s="3"/>
       <c r="K127" s="3"/>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -2244,7 +2210,7 @@
       <c r="J128" s="3"/>
       <c r="K128" s="3"/>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -2257,7 +2223,7 @@
       <c r="J129" s="3"/>
       <c r="K129" s="3"/>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -2270,7 +2236,7 @@
       <c r="J130" s="3"/>
       <c r="K130" s="3"/>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -2283,7 +2249,7 @@
       <c r="J131" s="3"/>
       <c r="K131" s="3"/>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -2296,7 +2262,7 @@
       <c r="J132" s="3"/>
       <c r="K132" s="3"/>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -2309,7 +2275,7 @@
       <c r="J133" s="3"/>
       <c r="K133" s="3"/>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -2322,7 +2288,7 @@
       <c r="J134" s="3"/>
       <c r="K134" s="3"/>
     </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -2335,7 +2301,7 @@
       <c r="J135" s="3"/>
       <c r="K135" s="3"/>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -2348,7 +2314,7 @@
       <c r="J136" s="3"/>
       <c r="K136" s="3"/>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -2361,7 +2327,7 @@
       <c r="J137" s="3"/>
       <c r="K137" s="3"/>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -2374,7 +2340,7 @@
       <c r="J138" s="3"/>
       <c r="K138" s="3"/>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -2387,7 +2353,7 @@
       <c r="J139" s="3"/>
       <c r="K139" s="3"/>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -2400,7 +2366,7 @@
       <c r="J140" s="3"/>
       <c r="K140" s="3"/>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -2413,7 +2379,7 @@
       <c r="J141" s="3"/>
       <c r="K141" s="3"/>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -2426,7 +2392,7 @@
       <c r="J142" s="3"/>
       <c r="K142" s="3"/>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -2439,7 +2405,7 @@
       <c r="J143" s="3"/>
       <c r="K143" s="3"/>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -2452,7 +2418,7 @@
       <c r="J144" s="3"/>
       <c r="K144" s="3"/>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -2465,7 +2431,7 @@
       <c r="J145" s="3"/>
       <c r="K145" s="3"/>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -2478,7 +2444,7 @@
       <c r="J146" s="3"/>
       <c r="K146" s="3"/>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -2491,7 +2457,7 @@
       <c r="J147" s="3"/>
       <c r="K147" s="3"/>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -2504,7 +2470,7 @@
       <c r="J148" s="3"/>
       <c r="K148" s="3"/>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -2517,7 +2483,7 @@
       <c r="J149" s="3"/>
       <c r="K149" s="3"/>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -2530,7 +2496,7 @@
       <c r="J150" s="3"/>
       <c r="K150" s="3"/>
     </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -2543,7 +2509,7 @@
       <c r="J151" s="3"/>
       <c r="K151" s="3"/>
     </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -2556,7 +2522,7 @@
       <c r="J152" s="3"/>
       <c r="K152" s="3"/>
     </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -2569,7 +2535,7 @@
       <c r="J153" s="3"/>
       <c r="K153" s="3"/>
     </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -2582,7 +2548,7 @@
       <c r="J154" s="3"/>
       <c r="K154" s="3"/>
     </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -2595,7 +2561,7 @@
       <c r="J155" s="3"/>
       <c r="K155" s="3"/>
     </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -2608,7 +2574,7 @@
       <c r="J156" s="3"/>
       <c r="K156" s="3"/>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -2621,7 +2587,7 @@
       <c r="J157" s="3"/>
       <c r="K157" s="3"/>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -2634,7 +2600,7 @@
       <c r="J158" s="3"/>
       <c r="K158" s="3"/>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -2647,7 +2613,7 @@
       <c r="J159" s="3"/>
       <c r="K159" s="3"/>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -2660,7 +2626,7 @@
       <c r="J160" s="3"/>
       <c r="K160" s="3"/>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -2673,7 +2639,7 @@
       <c r="J161" s="3"/>
       <c r="K161" s="3"/>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -2686,7 +2652,7 @@
       <c r="J162" s="3"/>
       <c r="K162" s="3"/>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -2699,7 +2665,7 @@
       <c r="J163" s="3"/>
       <c r="K163" s="3"/>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -2712,7 +2678,7 @@
       <c r="J164" s="3"/>
       <c r="K164" s="3"/>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -2725,7 +2691,7 @@
       <c r="J165" s="3"/>
       <c r="K165" s="3"/>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -2738,7 +2704,7 @@
       <c r="J166" s="3"/>
       <c r="K166" s="3"/>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -2751,7 +2717,7 @@
       <c r="J167" s="3"/>
       <c r="K167" s="3"/>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -2764,7 +2730,7 @@
       <c r="J168" s="3"/>
       <c r="K168" s="3"/>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -2777,7 +2743,7 @@
       <c r="J169" s="3"/>
       <c r="K169" s="3"/>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -2790,7 +2756,7 @@
       <c r="J170" s="3"/>
       <c r="K170" s="3"/>
     </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -2803,7 +2769,7 @@
       <c r="J171" s="3"/>
       <c r="K171" s="3"/>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -2816,7 +2782,7 @@
       <c r="J172" s="3"/>
       <c r="K172" s="3"/>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -2829,7 +2795,7 @@
       <c r="J173" s="3"/>
       <c r="K173" s="3"/>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -2842,7 +2808,7 @@
       <c r="J174" s="3"/>
       <c r="K174" s="3"/>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -2855,7 +2821,7 @@
       <c r="J175" s="3"/>
       <c r="K175" s="3"/>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -2868,7 +2834,7 @@
       <c r="J176" s="3"/>
       <c r="K176" s="3"/>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -2881,7 +2847,7 @@
       <c r="J177" s="3"/>
       <c r="K177" s="3"/>
     </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -2894,7 +2860,7 @@
       <c r="J178" s="3"/>
       <c r="K178" s="3"/>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -2907,7 +2873,7 @@
       <c r="J179" s="3"/>
       <c r="K179" s="3"/>
     </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -2920,7 +2886,7 @@
       <c r="J180" s="3"/>
       <c r="K180" s="3"/>
     </row>
-    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -2933,7 +2899,7 @@
       <c r="J181" s="3"/>
       <c r="K181" s="3"/>
     </row>
-    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -2946,7 +2912,7 @@
       <c r="J182" s="3"/>
       <c r="K182" s="3"/>
     </row>
-    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -2959,7 +2925,7 @@
       <c r="J183" s="3"/>
       <c r="K183" s="3"/>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -2972,7 +2938,7 @@
       <c r="J184" s="3"/>
       <c r="K184" s="3"/>
     </row>
-    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -2985,7 +2951,7 @@
       <c r="J185" s="3"/>
       <c r="K185" s="3"/>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -2998,7 +2964,7 @@
       <c r="J186" s="3"/>
       <c r="K186" s="3"/>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -3011,7 +2977,7 @@
       <c r="J187" s="3"/>
       <c r="K187" s="3"/>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -3024,7 +2990,7 @@
       <c r="J188" s="3"/>
       <c r="K188" s="3"/>
     </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -3037,7 +3003,7 @@
       <c r="J189" s="3"/>
       <c r="K189" s="3"/>
     </row>
-    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -3050,7 +3016,7 @@
       <c r="J190" s="3"/>
       <c r="K190" s="3"/>
     </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -3063,7 +3029,7 @@
       <c r="J191" s="3"/>
       <c r="K191" s="3"/>
     </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -3076,7 +3042,7 @@
       <c r="J192" s="3"/>
       <c r="K192" s="3"/>
     </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -3089,7 +3055,7 @@
       <c r="J193" s="3"/>
       <c r="K193" s="3"/>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -3102,7 +3068,7 @@
       <c r="J194" s="3"/>
       <c r="K194" s="3"/>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -3115,7 +3081,7 @@
       <c r="J195" s="3"/>
       <c r="K195" s="3"/>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -3128,7 +3094,7 @@
       <c r="J196" s="3"/>
       <c r="K196" s="3"/>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -3141,7 +3107,7 @@
       <c r="J197" s="3"/>
       <c r="K197" s="3"/>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -3154,7 +3120,7 @@
       <c r="J198" s="3"/>
       <c r="K198" s="3"/>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -3167,7 +3133,7 @@
       <c r="J199" s="3"/>
       <c r="K199" s="3"/>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -3182,122 +3148,114 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D500" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D500" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Easy,Medium,Hard"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F500" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F500" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Solved,Attempted,Revisit,Bookmarked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:3" ht="17.649999999999999" x14ac:dyDescent="0.5">
+      <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="6" t="n">
-        <f aca="false">COUNTA(Log!C2:C500)</f>
+      <c r="B3" s="5">
+        <f>COUNTA(Log!C2:C500)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIF(Log!F2:F500,"Solved")</f>
+      <c r="B4" s="5">
+        <f>COUNTIF(Log!F2:F500,"Solved")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF(Log!F2:F500,"Attempted")</f>
+      <c r="B5" s="5">
+        <f>COUNTIF(Log!F2:F500,"Attempted")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(Log!F2:F500,"Revisit")</f>
+      <c r="B6" s="5">
+        <f>COUNTIF(Log!F2:F500,"Revisit")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(Log!F2:F500,"Bookmarked")</f>
+      <c r="B7" s="5">
+        <f>COUNTIF(Log!F2:F500,"Bookmarked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIFS(Log!D2:D500,"Easy",Log!F2:F500,"Solved")</f>
+      <c r="B9" s="5">
+        <f>COUNTIFS(Log!D2:D500,"Easy",Log!F2:F500,"Solved")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="6" t="n">
-        <f aca="false">COUNTIFS(Log!D2:D500,"Medium",Log!F2:F500,"Solved")</f>
+      <c r="B10" s="5">
+        <f>COUNTIFS(Log!D2:D500,"Medium",Log!F2:F500,"Solved")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="6" t="n">
-        <f aca="false">COUNTIFS(Log!D2:D500,"Hard",Log!F2:F500,"Solved")</f>
+      <c r="B11" s="5">
+        <f>COUNTIFS(Log!D2:D500,"Hard",Log!F2:F500,"Solved")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(AVERAGEIF(Log!F2:F500,"Solved",Log!H2:H500),1),0)</f>
+      <c r="B13" s="5">
+        <f>IFERROR(ROUND(AVERAGEIF(Log!F2:F500,"Solved",Log!H2:H500),1),0)</f>
         <v>15</v>
       </c>
     </row>
@@ -3305,12 +3263,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>